<commit_message>
Add .gitattributes to normalize line endings (LF) and .gitignore for temp Office files
</commit_message>
<xml_diff>
--- a/Documents/Refined_proposal_ChatGPT.xlsx
+++ b/Documents/Refined_proposal_ChatGPT.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Business\Agentic Code\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Business\Agentic Code\Requirements_Tool_Local_AI\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56C648A2-CB94-4EF3-9C39-2FA91533C2C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C706D512-DA27-4AF2-A9CB-B43056D14A94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D17E0A88-1C2D-4A27-9B15-EB45CA17BC10}"/>
   </bookViews>
@@ -72,9 +72,6 @@
     <t>DeepSeek-R1:7b for content review and Gemma3:4b for structuring</t>
   </si>
   <si>
-    <t>List of functions/systems comprising the product</t>
-  </si>
-  <si>
     <t>Generic description of each function</t>
   </si>
   <si>
@@ -274,6 +271,9 @@
   </si>
   <si>
     <t>Author to Produce Initial version. Following review, AI can update this.</t>
+  </si>
+  <si>
+    <t>Product Name, Product Description, List of functions/systems comprising the product ,Hardware platform/Cloud platform/Software platform it will be based on for webapp, Android app, BFF and Backend plus Github link to save online in addtion to local</t>
   </si>
 </sst>
 </file>
@@ -731,7 +731,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="90" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="165" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -748,23 +748,23 @@
         <v>14</v>
       </c>
       <c r="F2" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="I2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="J2" s="6" t="s">
         <v>18</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>19</v>
       </c>
       <c r="L2" s="4"/>
       <c r="M2" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="60" x14ac:dyDescent="0.25">
@@ -772,35 +772,35 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C3" s="3">
         <v>1</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="H3" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="I3" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="J3" s="6" t="s">
         <v>25</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>26</v>
       </c>
       <c r="L3" s="5"/>
       <c r="M3" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="75" x14ac:dyDescent="0.25">
@@ -808,35 +808,35 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C4" s="3">
         <v>2</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="G4" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="H4" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="I4" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="J4" s="5" t="s">
         <v>34</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>35</v>
       </c>
       <c r="L4" s="6"/>
       <c r="M4" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="75" x14ac:dyDescent="0.25">
@@ -844,31 +844,31 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C5" s="3">
         <v>3</v>
       </c>
       <c r="D5" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="I5" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="J5" s="6" t="s">
         <v>41</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -876,31 +876,31 @@
         <v>5</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C6" s="3">
         <v>4</v>
       </c>
       <c r="D6" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="I6" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="J6" s="5" t="s">
         <v>48</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="60" x14ac:dyDescent="0.25">
@@ -908,31 +908,31 @@
         <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C7" s="3">
         <v>5</v>
       </c>
       <c r="D7" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F7" s="6" t="s">
+      <c r="G7" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="H7" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="I7" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="J7" s="6" t="s">
         <v>55</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="30" x14ac:dyDescent="0.25">
@@ -940,31 +940,31 @@
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C8" s="3">
         <v>6</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E8" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="F8" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="G8" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="H8" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="I8" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="J8" s="5" t="s">
         <v>62</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="45" x14ac:dyDescent="0.25">
@@ -972,31 +972,31 @@
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C9" s="3">
         <v>7</v>
       </c>
       <c r="D9" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="G9" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="H9" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="I9" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="H9" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="I9" s="6" t="s">
+      <c r="J9" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="J9" s="6" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="75" x14ac:dyDescent="0.25">
@@ -1004,31 +1004,31 @@
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C10" s="3">
         <v>8</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F10" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G10" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="H10" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="I10" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="J10" s="5" t="s">
         <v>75</v>
-      </c>
-      <c r="J10" s="5" t="s">
-        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Partial updates. Need to split the files beforehand
</commit_message>
<xml_diff>
--- a/Documents/Refined_proposal_ChatGPT.xlsx
+++ b/Documents/Refined_proposal_ChatGPT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Business\Agentic Code\Requirements_Tool_Local_AI\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8703169E-296A-40FC-8C89-A0932C32DF28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E67A901-EC41-46BF-90E0-5F750B213A81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{D17E0A88-1C2D-4A27-9B15-EB45CA17BC10}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="675" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="686" uniqueCount="306">
   <si>
     <t>Stage</t>
   </si>
@@ -499,13 +499,7 @@
     <t>If public facing android app is required?</t>
   </si>
   <si>
-    <t>D1.6.4</t>
-  </si>
-  <si>
     <t>If private android app is required?</t>
-  </si>
-  <si>
-    <t>D1.6.5</t>
   </si>
   <si>
     <t>BFF with public URL for normal and paid/premium users?</t>
@@ -917,6 +911,42 @@
   </si>
   <si>
     <t>LLM review will be marked AGRM as per tag legend when it has been created. If reviewed but no comments, it should still be marked AGRM since review was done. Tags to be done as per "Tag" colum. If review skipped, then don’t tag at all.</t>
+  </si>
+  <si>
+    <t>The entire history of Manual additions and AI reviews will be captured via tags in a json file. This will allow all choices to be replayed. Note that the "Tag" column includes a time field. So when manually entered, time of entry will be added here. If AI review is done, the time of AI review completion willl be here. If AI review accepted manually, that time of acceptance will be in this field. Same for edited or rejected.</t>
+  </si>
+  <si>
+    <t>D1.6.5.2</t>
+  </si>
+  <si>
+    <t>D1.6.5.3</t>
+  </si>
+  <si>
+    <t>D1.6.5.1</t>
+  </si>
+  <si>
+    <t>D1.6.4.1</t>
+  </si>
+  <si>
+    <t>S2</t>
+  </si>
+  <si>
+    <t>D4</t>
+  </si>
+  <si>
+    <t>LLM to be requested to generate a context diagram of entire product based on all the above content reviewed.</t>
+  </si>
+  <si>
+    <t>Context Diagram of Product</t>
+  </si>
+  <si>
+    <t>Max_functions_per_product = 10</t>
+  </si>
+  <si>
+    <t>The json file shall be automatically saved when clicking D5 autochecks.</t>
+  </si>
+  <si>
+    <t>There shall be a button to periodically save the json file.</t>
   </si>
 </sst>
 </file>
@@ -1446,7 +1476,7 @@
         <v>80</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>15</v>
@@ -1733,7 +1763,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{581B6C60-5ACF-4FEC-90F4-0E94D7E97E86}">
-  <dimension ref="A1:S71"/>
+  <dimension ref="A1:S72"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="2"/>
@@ -1749,7 +1779,7 @@
     <col min="12" max="12" width="22.28515625" style="2" customWidth="1"/>
     <col min="13" max="13" width="12.140625" style="2" customWidth="1"/>
     <col min="14" max="17" width="9.140625" style="2"/>
-    <col min="18" max="18" width="20.140625" style="2" customWidth="1"/>
+    <col min="18" max="18" width="22.7109375" style="2" customWidth="1"/>
     <col min="19" max="19" width="19.5703125" style="2" customWidth="1"/>
     <col min="20" max="16384" width="9.140625" style="2"/>
   </cols>
@@ -1780,19 +1810,19 @@
         <v>94</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
       <c r="L1" s="9" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="M1" s="9"/>
       <c r="R1" s="12" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="S1" s="12" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="90" x14ac:dyDescent="0.25">
@@ -1825,13 +1855,13 @@
         <v>S1_PRD_D1.1_(AorM)_(time)</v>
       </c>
       <c r="L2" s="10" t="s">
+        <v>282</v>
+      </c>
+      <c r="M2" s="10" t="s">
         <v>284</v>
       </c>
-      <c r="M2" s="10" t="s">
-        <v>286</v>
-      </c>
       <c r="R2" s="11" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="S2" s="11"/>
     </row>
@@ -1858,20 +1888,20 @@
         <v>98</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="I3" s="3" t="str">
         <f t="shared" ref="I3:I66" si="0">A3&amp;"_"&amp;B3&amp;"_"&amp;C3&amp;"_(AorM)_(time)"</f>
         <v>S1_PRD_D1.2_(AorM)_(time)</v>
       </c>
       <c r="L3" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="M3" s="10" t="s">
         <v>285</v>
       </c>
-      <c r="M3" s="10" t="s">
-        <v>287</v>
-      </c>
       <c r="R3" s="11" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="S3" s="11"/>
     </row>
@@ -1898,23 +1928,23 @@
         <v>92</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I4" s="3" t="str">
         <f t="shared" si="0"/>
         <v>S1_PRD_D1.2.1_(AorM)_(time)</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="M4" s="10" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="R4" s="11" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="S4" s="11" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="5" spans="1:19" ht="45" x14ac:dyDescent="0.25">
@@ -1940,20 +1970,20 @@
         <v>92</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I5" s="3" t="str">
         <f t="shared" si="0"/>
         <v>S1_PRD_D1.2.2_(AorM)_(time)</v>
       </c>
       <c r="L5" s="10" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="M5" s="10" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="R5" s="11" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="S5" s="11"/>
     </row>
@@ -1987,13 +2017,13 @@
         <v>S1_PRD_D1.2.3_(AorM)_(time)</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="M6" s="10" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="R6" s="11" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="S6" s="11"/>
     </row>
@@ -2020,20 +2050,20 @@
         <v>92</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I7" s="3" t="str">
         <f t="shared" si="0"/>
         <v>S1_PRD_D1.2.3.1_(AorM)_(time)</v>
       </c>
       <c r="L7" s="10" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="M7" s="10" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="R7" s="11" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="S7" s="11"/>
     </row>
@@ -2060,17 +2090,17 @@
         <v>92</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I8" s="3" t="str">
         <f t="shared" si="0"/>
         <v>S1_PRD_D1.2.3.2_(AorM)_(time)</v>
       </c>
       <c r="R8" s="11" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="S8" s="11" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
     </row>
     <row r="9" spans="1:19" ht="120" x14ac:dyDescent="0.25">
@@ -2096,18 +2126,18 @@
         <v>92</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I9" s="3" t="str">
         <f t="shared" si="0"/>
         <v>S1_PRD_D1.2.3.3_(AorM)_(time)</v>
       </c>
       <c r="R9" s="11" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="S9" s="11"/>
     </row>
-    <row r="10" spans="1:19" ht="60" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:19" ht="285" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>82</v>
       </c>
@@ -2130,11 +2160,14 @@
         <v>92</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I10" s="3" t="str">
         <f t="shared" si="0"/>
         <v>S1_PRD_D1.2.3.4_(AorM)_(time)</v>
+      </c>
+      <c r="R10" s="11" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="30" x14ac:dyDescent="0.25">
@@ -2160,14 +2193,17 @@
         <v>92</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I11" s="3" t="str">
         <f t="shared" si="0"/>
         <v>S1_PRD_D1.2.3.5_(AorM)_(time)</v>
       </c>
-    </row>
-    <row r="12" spans="1:19" ht="30" x14ac:dyDescent="0.25">
+      <c r="R11" s="11" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>82</v>
       </c>
@@ -2190,11 +2226,14 @@
         <v>92</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I12" s="3" t="str">
         <f t="shared" si="0"/>
         <v>S1_PRD_D1.2.3.6_(AorM)_(time)</v>
+      </c>
+      <c r="R12" s="11" t="s">
+        <v>304</v>
       </c>
     </row>
     <row r="13" spans="1:19" ht="45" x14ac:dyDescent="0.25">
@@ -2208,7 +2247,7 @@
         <v>87</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>128</v>
@@ -2220,11 +2259,14 @@
         <v>98</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="I13" s="3" t="str">
         <f t="shared" si="0"/>
         <v>S1_PRD_D1.3_(AorM)_(time)</v>
+      </c>
+      <c r="R13" s="11" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="14" spans="1:19" ht="30" x14ac:dyDescent="0.25">
@@ -2280,7 +2322,7 @@
         <v>92</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I15" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2340,7 +2382,7 @@
         <v>92</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I17" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2355,7 +2397,7 @@
         <v>84</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>139</v>
@@ -2385,7 +2427,7 @@
         <v>84</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>141</v>
@@ -2400,7 +2442,7 @@
         <v>92</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I19" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2415,7 +2457,7 @@
         <v>84</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>142</v>
@@ -2430,7 +2472,7 @@
         <v>92</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I20" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2475,7 +2517,7 @@
         <v>84</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="D22" s="3" t="s">
         <v>151</v>
@@ -2490,7 +2532,7 @@
         <v>92</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I22" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2505,14 +2547,14 @@
         <v>84</v>
       </c>
       <c r="C23" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="D23" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="E23" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="E23" s="3" t="s">
-        <v>173</v>
-      </c>
       <c r="F23" s="3" t="s">
         <v>92</v>
       </c>
@@ -2520,7 +2562,7 @@
         <v>92</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I23" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2535,14 +2577,14 @@
         <v>84</v>
       </c>
       <c r="C24" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="E24" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="E24" s="3" t="s">
-        <v>174</v>
-      </c>
       <c r="F24" s="3" t="s">
         <v>92</v>
       </c>
@@ -2550,7 +2592,7 @@
         <v>92</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I24" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2565,7 +2607,7 @@
         <v>84</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>152</v>
@@ -2580,7 +2622,7 @@
         <v>92</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I25" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2595,14 +2637,14 @@
         <v>84</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="D26" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="E26" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="E26" s="3" t="s">
-        <v>173</v>
-      </c>
       <c r="F26" s="3" t="s">
         <v>92</v>
       </c>
@@ -2610,7 +2652,7 @@
         <v>92</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I26" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2625,14 +2667,14 @@
         <v>84</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="D27" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="E27" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="E27" s="3" t="s">
-        <v>174</v>
-      </c>
       <c r="F27" s="3" t="s">
         <v>92</v>
       </c>
@@ -2640,7 +2682,7 @@
         <v>92</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I27" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2655,7 +2697,7 @@
         <v>84</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>155</v>
@@ -2670,7 +2712,7 @@
         <v>92</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I28" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2685,13 +2727,13 @@
         <v>84</v>
       </c>
       <c r="C29" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="D29" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="D29" s="3" t="s">
-        <v>182</v>
-      </c>
       <c r="E29" s="3" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>92</v>
@@ -2700,7 +2742,7 @@
         <v>92</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I29" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2715,13 +2757,13 @@
         <v>84</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="F30" s="3" t="s">
         <v>92</v>
@@ -2730,7 +2772,7 @@
         <v>92</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I30" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2745,13 +2787,13 @@
         <v>84</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>157</v>
+        <v>298</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>155</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>92</v>
@@ -2760,11 +2802,11 @@
         <v>92</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I31" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>S1_PRD_D1.6.4_(AorM)_(time)</v>
+        <v>S1_PRD_D1.6.4.1_(AorM)_(time)</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="30" x14ac:dyDescent="0.25">
@@ -2775,13 +2817,13 @@
         <v>84</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>92</v>
@@ -2790,7 +2832,7 @@
         <v>92</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I32" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2805,13 +2847,13 @@
         <v>84</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>92</v>
@@ -2820,7 +2862,7 @@
         <v>92</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I33" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2835,14 +2877,14 @@
         <v>84</v>
       </c>
       <c r="C34" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E34" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="D34" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>161</v>
-      </c>
       <c r="F34" s="3" t="s">
         <v>92</v>
       </c>
@@ -2850,11 +2892,11 @@
         <v>92</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I34" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>S1_PRD_D1.6.5_(AorM)_(time)</v>
+        <v>S1_PRD_D1.6.5.1_(AorM)_(time)</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
@@ -2865,13 +2907,13 @@
         <v>84</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>176</v>
+        <v>295</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>92</v>
@@ -2880,11 +2922,11 @@
         <v>92</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I35" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>S1_PRD_D1.6.2.2_(AorM)_(time)</v>
+        <v>S1_PRD_D1.6.5.2_(AorM)_(time)</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
@@ -2895,14 +2937,14 @@
         <v>84</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>177</v>
+        <v>296</v>
       </c>
       <c r="D36" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="E36" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="E36" s="3" t="s">
-        <v>174</v>
-      </c>
       <c r="F36" s="3" t="s">
         <v>92</v>
       </c>
@@ -2910,11 +2952,11 @@
         <v>92</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I36" s="3" t="str">
         <f t="shared" si="0"/>
-        <v>S1_PRD_D1.6.2.3_(AorM)_(time)</v>
+        <v>S1_PRD_D1.6.5.3_(AorM)_(time)</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -2925,13 +2967,13 @@
         <v>84</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="F37" s="3" t="s">
         <v>92</v>
@@ -2940,7 +2982,7 @@
         <v>92</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I37" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2955,13 +2997,13 @@
         <v>84</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="F38" s="3" t="s">
         <v>92</v>
@@ -2970,7 +3012,7 @@
         <v>92</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I38" s="3" t="str">
         <f t="shared" si="0"/>
@@ -2985,14 +3027,14 @@
         <v>84</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D39" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="E39" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="E39" s="3" t="s">
-        <v>174</v>
-      </c>
       <c r="F39" s="3" t="s">
         <v>92</v>
       </c>
@@ -3000,7 +3042,7 @@
         <v>92</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I39" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3015,13 +3057,13 @@
         <v>84</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F40" s="3" t="s">
         <v>92</v>
@@ -3030,7 +3072,7 @@
         <v>92</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I40" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3045,13 +3087,13 @@
         <v>84</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="F41" s="3" t="s">
         <v>92</v>
@@ -3060,7 +3102,7 @@
         <v>92</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I41" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3075,13 +3117,13 @@
         <v>84</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>92</v>
@@ -3090,7 +3132,7 @@
         <v>92</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I42" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3105,13 +3147,13 @@
         <v>84</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F43" s="3" t="s">
         <v>92</v>
@@ -3120,7 +3162,7 @@
         <v>92</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I43" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3135,13 +3177,13 @@
         <v>84</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="F44" s="3" t="s">
         <v>92</v>
@@ -3150,7 +3192,7 @@
         <v>92</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I44" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3165,14 +3207,14 @@
         <v>84</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D45" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="E45" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="E45" s="3" t="s">
-        <v>174</v>
-      </c>
       <c r="F45" s="3" t="s">
         <v>92</v>
       </c>
@@ -3180,7 +3222,7 @@
         <v>92</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I45" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3195,13 +3237,13 @@
         <v>84</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E46" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F46" s="3" t="s">
         <v>92</v>
@@ -3210,7 +3252,7 @@
         <v>92</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I46" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3225,13 +3267,13 @@
         <v>84</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E47" s="3" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="F47" s="3" t="s">
         <v>92</v>
@@ -3240,7 +3282,7 @@
         <v>92</v>
       </c>
       <c r="H47" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I47" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3255,13 +3297,13 @@
         <v>84</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="F48" s="3" t="s">
         <v>92</v>
@@ -3270,7 +3312,7 @@
         <v>92</v>
       </c>
       <c r="H48" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I48" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3285,13 +3327,13 @@
         <v>84</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="F49" s="3" t="s">
         <v>92</v>
@@ -3300,7 +3342,7 @@
         <v>92</v>
       </c>
       <c r="H49" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I49" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3315,14 +3357,14 @@
         <v>84</v>
       </c>
       <c r="C50" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="E50" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="D50" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="E50" s="3" t="s">
-        <v>205</v>
-      </c>
       <c r="F50" s="3" t="s">
         <v>92</v>
       </c>
@@ -3330,7 +3372,7 @@
         <v>92</v>
       </c>
       <c r="H50" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I50" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3345,13 +3387,13 @@
         <v>84</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="F51" s="3" t="s">
         <v>92</v>
@@ -3360,7 +3402,7 @@
         <v>92</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I51" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3375,13 +3417,13 @@
         <v>84</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="F52" s="3" t="s">
         <v>98</v>
@@ -3405,13 +3447,13 @@
         <v>84</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="F53" s="3" t="s">
         <v>92</v>
@@ -3420,7 +3462,7 @@
         <v>92</v>
       </c>
       <c r="H53" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I53" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3435,13 +3477,13 @@
         <v>84</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="F54" s="3" t="s">
         <v>92</v>
@@ -3450,7 +3492,7 @@
         <v>92</v>
       </c>
       <c r="H54" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I54" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3465,14 +3507,14 @@
         <v>84</v>
       </c>
       <c r="C55" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="D55" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="D55" s="3" t="s">
+      <c r="E55" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="E55" s="3" t="s">
-        <v>221</v>
-      </c>
       <c r="F55" s="3" t="s">
         <v>92</v>
       </c>
@@ -3480,7 +3522,7 @@
         <v>92</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I55" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3495,14 +3537,14 @@
         <v>84</v>
       </c>
       <c r="C56" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="E56" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="D56" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="E56" s="3" t="s">
-        <v>220</v>
-      </c>
       <c r="F56" s="3" t="s">
         <v>92</v>
       </c>
@@ -3510,7 +3552,7 @@
         <v>92</v>
       </c>
       <c r="H56" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I56" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3525,13 +3567,13 @@
         <v>84</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E57" s="3" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="F57" s="3" t="s">
         <v>92</v>
@@ -3540,7 +3582,7 @@
         <v>92</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I57" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3555,14 +3597,14 @@
         <v>84</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D58" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="E58" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="E58" s="3" t="s">
-        <v>225</v>
-      </c>
       <c r="F58" s="3" t="s">
         <v>92</v>
       </c>
@@ -3570,7 +3612,7 @@
         <v>92</v>
       </c>
       <c r="H58" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I58" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3585,13 +3627,13 @@
         <v>84</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="F59" s="3" t="s">
         <v>92</v>
@@ -3600,7 +3642,7 @@
         <v>92</v>
       </c>
       <c r="H59" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I59" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3615,14 +3657,14 @@
         <v>84</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D60" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="E60" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="E60" s="3" t="s">
-        <v>232</v>
-      </c>
       <c r="F60" s="3" t="s">
         <v>92</v>
       </c>
@@ -3630,7 +3672,7 @@
         <v>92</v>
       </c>
       <c r="H60" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I60" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3645,13 +3687,13 @@
         <v>84</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="F61" s="3" t="s">
         <v>92</v>
@@ -3660,7 +3702,7 @@
         <v>92</v>
       </c>
       <c r="H61" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I61" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3675,14 +3717,14 @@
         <v>84</v>
       </c>
       <c r="C62" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="E62" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="D62" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="E62" s="3" t="s">
-        <v>243</v>
-      </c>
       <c r="F62" s="3" t="s">
         <v>92</v>
       </c>
@@ -3690,7 +3732,7 @@
         <v>92</v>
       </c>
       <c r="H62" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="I62" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3705,13 +3747,13 @@
         <v>84</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F63" s="3" t="s">
         <v>98</v>
@@ -3735,13 +3777,13 @@
         <v>84</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="F64" s="3" t="s">
         <v>98</v>
@@ -3750,7 +3792,7 @@
         <v>92</v>
       </c>
       <c r="H64" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I64" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3765,13 +3807,13 @@
         <v>84</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="F65" s="3" t="s">
         <v>98</v>
@@ -3780,7 +3822,7 @@
         <v>92</v>
       </c>
       <c r="H65" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I65" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3795,10 +3837,10 @@
         <v>84</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="E66" s="3"/>
       <c r="F66" s="3" t="s">
@@ -3808,7 +3850,7 @@
         <v>92</v>
       </c>
       <c r="H66" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I66" s="3" t="str">
         <f t="shared" si="0"/>
@@ -3823,10 +3865,10 @@
         <v>84</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="E67" s="3"/>
       <c r="F67" s="3" t="s">
@@ -3836,7 +3878,7 @@
         <v>92</v>
       </c>
       <c r="H67" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I67" s="3" t="str">
         <f t="shared" ref="I67:I71" si="1">A67&amp;"_"&amp;B67&amp;"_"&amp;C67&amp;"_(AorM)_(time)"</f>
@@ -3851,10 +3893,10 @@
         <v>84</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="E68" s="3"/>
       <c r="F68" s="3" t="s">
@@ -3864,7 +3906,7 @@
         <v>92</v>
       </c>
       <c r="H68" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I68" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3879,10 +3921,10 @@
         <v>84</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="E69" s="3"/>
       <c r="F69" s="3" t="s">
@@ -3892,7 +3934,7 @@
         <v>92</v>
       </c>
       <c r="H69" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I69" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3907,10 +3949,10 @@
         <v>84</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="E70" s="3"/>
       <c r="F70" s="3" t="s">
@@ -3920,7 +3962,7 @@
         <v>92</v>
       </c>
       <c r="H70" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I70" s="3" t="str">
         <f t="shared" si="1"/>
@@ -3935,10 +3977,10 @@
         <v>84</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="E71" s="3"/>
       <c r="F71" s="3" t="s">
@@ -3948,12 +3990,37 @@
         <v>92</v>
       </c>
       <c r="H71" s="3" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="I71" s="3" t="str">
         <f t="shared" si="1"/>
         <v>S1_PRD_D5.x.x_(AorM)_(time)</v>
       </c>
+    </row>
+    <row r="72" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A72" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="B72" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="F72" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="G72" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H72" s="3"/>
+      <c r="I72" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>